<commit_message>
Cleaned all the sheets in Freshmart
</commit_message>
<xml_diff>
--- a/Excel/Project/Freshmart/Cleaned/Cleaned_FreshMart_Products.xlsx
+++ b/Excel/Project/Freshmart/Cleaned/Cleaned_FreshMart_Products.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnudipCOA\Desktop\Rithiha\Excel\Project\Freshmart\Cleaned\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/AB6FF4EDD41B64DB/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB82856A-C08B-4A43-947F-4537C6ACAE90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{65343440-51A6-4FEA-8C41-AE7A82F7F102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{649E3FE4-4A34-4549-B7B8-130120CE0B53}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{0642A12E-5FF2-42FC-BE12-DFEBADDDAB76}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0642A12E-5FF2-42FC-BE12-DFEBADDDAB76}"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
+    <sheet name="Data_profiling" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1200" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1226" uniqueCount="493">
   <si>
     <t>Active</t>
   </si>
@@ -1485,13 +1484,46 @@
   </si>
   <si>
     <t>Product_ID</t>
+  </si>
+  <si>
+    <t>Column_name</t>
+  </si>
+  <si>
+    <t>Issue_Description</t>
+  </si>
+  <si>
+    <t>Columns_affected</t>
+  </si>
+  <si>
+    <t>Changes_done</t>
+  </si>
+  <si>
+    <t>Blanks</t>
+  </si>
+  <si>
+    <t>Highlighted</t>
+  </si>
+  <si>
+    <t>Different Formats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed using Mapping </t>
+  </si>
+  <si>
+    <t>Inactive</t>
+  </si>
+  <si>
+    <t>In-active</t>
+  </si>
+  <si>
+    <t>Status2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1511,8 +1543,16 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1523,6 +1563,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
         <bgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1538,43 +1584,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F4E78"/>
-          <bgColor rgb="FF1F4E78"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="13">
     <dxf>
       <font>
         <b val="0"/>
@@ -1592,6 +1616,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <font>
@@ -1775,6 +1800,49 @@
         <scheme val="none"/>
       </font>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF1F4E78"/>
+          <bgColor rgb="FF1F4E78"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1789,19 +1857,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AECD1D58-74B5-4A3D-B534-93BFB62C73B5}" name="Table1" displayName="Table1" ref="A1:J151" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:J151" xr:uid="{AECD1D58-74B5-4A3D-B534-93BFB62C73B5}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{6A5350A9-9968-46C4-B3C6-130C09F8864F}" name="Product_ID" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{446D5102-4E26-4B3E-833E-E8D475B7200E}" name="Product_Name" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{D675CC66-306E-43D8-A726-962F9B7AA5B3}" name="Category" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{64872C1B-D6D8-4BA3-8DD2-65F807836053}" name="Subcategory" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{6E05A3A4-43FA-4C17-BB11-D9DD1F3E38DB}" name="Brand" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{38E1FB40-4D9A-4FAF-8FEE-A85E5629E637}" name="Cost_Price" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{7E9EF3A0-D0B3-4757-A03B-E289B886FDAB}" name="Selling_Price" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{DA6166B7-8385-47D1-918A-7FAE74B5AD53}" name="Supplier_ID" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{B224FB3F-E267-49FA-9477-2D817BC1169B}" name="Season" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{2BDD2FBE-CCEC-4E3E-A1BA-D37693288B8C}" name="Status" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AECD1D58-74B5-4A3D-B534-93BFB62C73B5}" name="Table1" displayName="Table1" ref="A1:K151" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A1:K151" xr:uid="{AECD1D58-74B5-4A3D-B534-93BFB62C73B5}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{6A5350A9-9968-46C4-B3C6-130C09F8864F}" name="Product_ID" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{446D5102-4E26-4B3E-833E-E8D475B7200E}" name="Product_Name" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{D675CC66-306E-43D8-A726-962F9B7AA5B3}" name="Category" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{64872C1B-D6D8-4BA3-8DD2-65F807836053}" name="Subcategory" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{6E05A3A4-43FA-4C17-BB11-D9DD1F3E38DB}" name="Brand" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{38E1FB40-4D9A-4FAF-8FEE-A85E5629E637}" name="Cost_Price" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{7E9EF3A0-D0B3-4757-A03B-E289B886FDAB}" name="Selling_Price" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{DA6166B7-8385-47D1-918A-7FAE74B5AD53}" name="Supplier_ID" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{B224FB3F-E267-49FA-9477-2D817BC1169B}" name="Season" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{62198AEC-6FF5-4DF4-B62B-5BEA2F741B44}" name="Status" dataDxfId="0">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="10" xr3:uid="{2BDD2FBE-CCEC-4E3E-A1BA-D37693288B8C}" name="Status2" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2124,22 +2195,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E349CBF3-A630-420B-9415-5BFE31CB5CE5}">
-  <dimension ref="A1:J151"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K151"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="19" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" customWidth="1"/>
+    <col min="6" max="6" width="14.26953125" customWidth="1"/>
+    <col min="7" max="7" width="16.54296875" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="11" customWidth="1"/>
+    <col min="10" max="10" width="22.26953125" customWidth="1"/>
+    <col min="11" max="11" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>481</v>
       </c>
@@ -2170,8 +2242,11 @@
       <c r="J1" s="3" t="s">
         <v>472</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="3" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>471</v>
       </c>
@@ -2199,11 +2274,15 @@
       <c r="I2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J2" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J2" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>468</v>
       </c>
@@ -2231,11 +2310,15 @@
       <c r="I3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J3" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>466</v>
       </c>
@@ -2263,11 +2346,15 @@
       <c r="I4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J4" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>464</v>
       </c>
@@ -2295,11 +2382,15 @@
       <c r="I5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J5" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>462</v>
       </c>
@@ -2327,11 +2418,15 @@
       <c r="I6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J6" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>460</v>
       </c>
@@ -2359,11 +2454,15 @@
       <c r="I7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K7" s="1" t="s">
         <v>458</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>457</v>
       </c>
@@ -2391,11 +2490,15 @@
       <c r="I8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J8" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>455</v>
       </c>
@@ -2423,11 +2526,15 @@
       <c r="I9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J9" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>453</v>
       </c>
@@ -2455,11 +2562,15 @@
       <c r="I10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J10" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>449</v>
       </c>
@@ -2487,11 +2598,15 @@
       <c r="I11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J11" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J11" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>444</v>
       </c>
@@ -2519,11 +2634,15 @@
       <c r="I12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J12" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J12" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>441</v>
       </c>
@@ -2551,11 +2670,15 @@
       <c r="I13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J13" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J13" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>437</v>
       </c>
@@ -2583,11 +2706,15 @@
       <c r="I14" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J14" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>435</v>
       </c>
@@ -2615,11 +2742,15 @@
       <c r="I15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J15" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J15" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>433</v>
       </c>
@@ -2647,11 +2778,15 @@
       <c r="I16" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J16" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J16" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>431</v>
       </c>
@@ -2679,11 +2814,15 @@
       <c r="I17" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="J17" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K17" s="1" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>428</v>
       </c>
@@ -2711,11 +2850,15 @@
       <c r="I18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J18" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J18" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>424</v>
       </c>
@@ -2743,11 +2886,15 @@
       <c r="I19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J19" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J19" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>421</v>
       </c>
@@ -2775,11 +2922,15 @@
       <c r="I20" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J20" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J20" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>418</v>
       </c>
@@ -2807,11 +2958,15 @@
       <c r="I21" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J21" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J21" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>416</v>
       </c>
@@ -2839,11 +2994,15 @@
       <c r="I22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J22" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J22" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>413</v>
       </c>
@@ -2871,11 +3030,15 @@
       <c r="I23" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J23" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J23" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>411</v>
       </c>
@@ -2888,7 +3051,7 @@
       <c r="D24" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="E24" s="1"/>
+      <c r="E24" s="5"/>
       <c r="F24" s="2">
         <v>266.10000000000002</v>
       </c>
@@ -2901,11 +3064,15 @@
       <c r="I24" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J24" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J24" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>407</v>
       </c>
@@ -2933,11 +3100,15 @@
       <c r="I25" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J25" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J25" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>402</v>
       </c>
@@ -2965,11 +3136,15 @@
       <c r="I26" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J26" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>400</v>
       </c>
@@ -2997,11 +3172,15 @@
       <c r="I27" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J27" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J27" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>398</v>
       </c>
@@ -3029,11 +3208,15 @@
       <c r="I28" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J28" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J28" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>395</v>
       </c>
@@ -3061,11 +3244,15 @@
       <c r="I29" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J29" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J29" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>392</v>
       </c>
@@ -3093,11 +3280,15 @@
       <c r="I30" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J30" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J30" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>389</v>
       </c>
@@ -3125,11 +3316,15 @@
       <c r="I31" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J31" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J31" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>386</v>
       </c>
@@ -3157,11 +3352,15 @@
       <c r="I32" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J32" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J32" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>384</v>
       </c>
@@ -3189,11 +3388,15 @@
       <c r="I33" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J33" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J33" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>381</v>
       </c>
@@ -3221,11 +3424,15 @@
       <c r="I34" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J34" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J34" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>377</v>
       </c>
@@ -3253,11 +3460,15 @@
       <c r="I35" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J35" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J35" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>374</v>
       </c>
@@ -3285,11 +3496,15 @@
       <c r="I36" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J36" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J36" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>369</v>
       </c>
@@ -3317,11 +3532,15 @@
       <c r="I37" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J37" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J37" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>366</v>
       </c>
@@ -3349,11 +3568,15 @@
       <c r="I38" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J38" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J38" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>362</v>
       </c>
@@ -3381,11 +3604,15 @@
       <c r="I39" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J39" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J39" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K39" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>359</v>
       </c>
@@ -3413,11 +3640,15 @@
       <c r="I40" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J40" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J40" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>357</v>
       </c>
@@ -3445,11 +3676,15 @@
       <c r="I41" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J41" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J41" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>355</v>
       </c>
@@ -3477,11 +3712,15 @@
       <c r="I42" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J42" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J42" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K42" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>353</v>
       </c>
@@ -3509,11 +3748,15 @@
       <c r="I43" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J43" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J43" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>349</v>
       </c>
@@ -3541,11 +3784,15 @@
       <c r="I44" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J44" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J44" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K44" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>347</v>
       </c>
@@ -3573,11 +3820,15 @@
       <c r="I45" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J45" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J45" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K45" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>344</v>
       </c>
@@ -3605,11 +3856,15 @@
       <c r="I46" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J46" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J46" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>340</v>
       </c>
@@ -3637,11 +3892,15 @@
       <c r="I47" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J47" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J47" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K47" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>335</v>
       </c>
@@ -3669,11 +3928,15 @@
       <c r="I48" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J48" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J48" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K48" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>333</v>
       </c>
@@ -3698,12 +3961,16 @@
       <c r="H49" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="I49" s="1"/>
-      <c r="J49" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I49" s="5"/>
+      <c r="J49" s="5" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K49" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>330</v>
       </c>
@@ -3731,11 +3998,15 @@
       <c r="I50" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J50" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J50" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K50" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>327</v>
       </c>
@@ -3763,11 +4034,15 @@
       <c r="I51" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J51" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J51" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K51" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>325</v>
       </c>
@@ -3795,11 +4070,15 @@
       <c r="I52" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J52" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J52" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>323</v>
       </c>
@@ -3827,11 +4106,15 @@
       <c r="I53" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J53" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J53" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K53" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>321</v>
       </c>
@@ -3859,11 +4142,15 @@
       <c r="I54" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J54" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J54" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>319</v>
       </c>
@@ -3891,11 +4178,15 @@
       <c r="I55" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J55" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J55" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>316</v>
       </c>
@@ -3923,11 +4214,15 @@
       <c r="I56" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J56" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J56" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>312</v>
       </c>
@@ -3955,11 +4250,15 @@
       <c r="I57" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J57" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J57" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K57" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>307</v>
       </c>
@@ -3987,11 +4286,15 @@
       <c r="I58" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J58" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J58" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K58" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>301</v>
       </c>
@@ -4019,11 +4322,15 @@
       <c r="I59" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J59" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J59" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K59" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>299</v>
       </c>
@@ -4051,11 +4358,15 @@
       <c r="I60" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J60" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J60" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K60" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>297</v>
       </c>
@@ -4068,7 +4379,7 @@
       <c r="D61" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="E61" s="1"/>
+      <c r="E61" s="5"/>
       <c r="F61" s="2">
         <v>54.25</v>
       </c>
@@ -4081,11 +4392,15 @@
       <c r="I61" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J61" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J61" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K61" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>295</v>
       </c>
@@ -4113,11 +4428,15 @@
       <c r="I62" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J62" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J62" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K62" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>292</v>
       </c>
@@ -4145,11 +4464,15 @@
       <c r="I63" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J63" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J63" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K63" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>288</v>
       </c>
@@ -4177,11 +4500,15 @@
       <c r="I64" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J64" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J64" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K64" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>285</v>
       </c>
@@ -4209,11 +4536,15 @@
       <c r="I65" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J65" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J65" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K65" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>282</v>
       </c>
@@ -4241,11 +4572,15 @@
       <c r="I66" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J66" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J66" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>278</v>
       </c>
@@ -4273,11 +4608,15 @@
       <c r="I67" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J67" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J67" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K67" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>275</v>
       </c>
@@ -4305,11 +4644,15 @@
       <c r="I68" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J68" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J68" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K68" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>272</v>
       </c>
@@ -4337,11 +4680,15 @@
       <c r="I69" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J69" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J69" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K69" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>269</v>
       </c>
@@ -4369,11 +4716,15 @@
       <c r="I70" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J70" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J70" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K70" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>264</v>
       </c>
@@ -4401,11 +4752,15 @@
       <c r="I71" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J71" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J71" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>261</v>
       </c>
@@ -4433,11 +4788,15 @@
       <c r="I72" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J72" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J72" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>259</v>
       </c>
@@ -4465,11 +4824,15 @@
       <c r="I73" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J73" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J73" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>257</v>
       </c>
@@ -4497,11 +4860,15 @@
       <c r="I74" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J74" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J74" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K74" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>254</v>
       </c>
@@ -4529,11 +4896,15 @@
       <c r="I75" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J75" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J75" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K75" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>251</v>
       </c>
@@ -4561,11 +4932,15 @@
       <c r="I76" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J76" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J76" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>250</v>
       </c>
@@ -4593,11 +4968,15 @@
       <c r="I77" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J77" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J77" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K77" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>246</v>
       </c>
@@ -4625,11 +5004,15 @@
       <c r="I78" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J78" s="1" t="s">
+      <c r="J78" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Inactive</v>
+      </c>
+      <c r="K78" s="1" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>241</v>
       </c>
@@ -4657,11 +5040,15 @@
       <c r="I79" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J79" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J79" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K79" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>238</v>
       </c>
@@ -4686,12 +5073,16 @@
       <c r="H80" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I80" s="1"/>
-      <c r="J80" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I80" s="5"/>
+      <c r="J80" s="5" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K80" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>235</v>
       </c>
@@ -4719,11 +5110,15 @@
       <c r="I81" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J81" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J81" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K81" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>231</v>
       </c>
@@ -4751,11 +5146,15 @@
       <c r="I82" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J82" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J82" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K82" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>225</v>
       </c>
@@ -4783,11 +5182,15 @@
       <c r="I83" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J83" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J83" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K83" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>223</v>
       </c>
@@ -4815,11 +5218,15 @@
       <c r="I84" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J84" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J84" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K84" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>219</v>
       </c>
@@ -4847,11 +5254,15 @@
       <c r="I85" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J85" s="1" t="s">
+      <c r="J85" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Inactive</v>
+      </c>
+      <c r="K85" s="1" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>215</v>
       </c>
@@ -4879,11 +5290,15 @@
       <c r="I86" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J86" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J86" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K86" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>213</v>
       </c>
@@ -4911,11 +5326,15 @@
       <c r="I87" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J87" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J87" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K87" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>210</v>
       </c>
@@ -4943,11 +5362,15 @@
       <c r="I88" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J88" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J88" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K88" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>208</v>
       </c>
@@ -4975,11 +5398,15 @@
       <c r="I89" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J89" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J89" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K89" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>205</v>
       </c>
@@ -5007,11 +5434,15 @@
       <c r="I90" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J90" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J90" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K90" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>202</v>
       </c>
@@ -5039,11 +5470,15 @@
       <c r="I91" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J91" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J91" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K91" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>200</v>
       </c>
@@ -5071,11 +5506,15 @@
       <c r="I92" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J92" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J92" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K92" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>196</v>
       </c>
@@ -5103,11 +5542,15 @@
       <c r="I93" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J93" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J93" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K93" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>192</v>
       </c>
@@ -5135,11 +5578,15 @@
       <c r="I94" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J94" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J94" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K94" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>189</v>
       </c>
@@ -5152,7 +5599,7 @@
       <c r="D95" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="E95" s="1"/>
+      <c r="E95" s="5"/>
       <c r="F95" s="2">
         <v>250.69</v>
       </c>
@@ -5165,11 +5612,15 @@
       <c r="I95" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J95" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J95" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K95" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>186</v>
       </c>
@@ -5197,11 +5648,15 @@
       <c r="I96" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J96" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J96" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K96" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>184</v>
       </c>
@@ -5229,11 +5684,15 @@
       <c r="I97" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J97" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J97" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K97" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>182</v>
       </c>
@@ -5261,11 +5720,15 @@
       <c r="I98" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J98" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J98" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K98" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>180</v>
       </c>
@@ -5278,7 +5741,7 @@
       <c r="D99" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="E99" s="1"/>
+      <c r="E99" s="5"/>
       <c r="F99" s="2">
         <v>69.09</v>
       </c>
@@ -5291,11 +5754,15 @@
       <c r="I99" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J99" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J99" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K99" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>177</v>
       </c>
@@ -5323,11 +5790,15 @@
       <c r="I100" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J100" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J100" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K100" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>175</v>
       </c>
@@ -5355,11 +5826,15 @@
       <c r="I101" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J101" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J101" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K101" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>172</v>
       </c>
@@ -5387,11 +5862,15 @@
       <c r="I102" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J102" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J102" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K102" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>170</v>
       </c>
@@ -5419,11 +5898,15 @@
       <c r="I103" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J103" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J103" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K103" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>168</v>
       </c>
@@ -5451,11 +5934,15 @@
       <c r="I104" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J104" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J104" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K104" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>164</v>
       </c>
@@ -5483,11 +5970,15 @@
       <c r="I105" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J105" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J105" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K105" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>158</v>
       </c>
@@ -5515,11 +6006,15 @@
       <c r="I106" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J106" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J106" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K106" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>156</v>
       </c>
@@ -5547,11 +6042,15 @@
       <c r="I107" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J107" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J107" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K107" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>153</v>
       </c>
@@ -5579,11 +6078,15 @@
       <c r="I108" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J108" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J108" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K108" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>151</v>
       </c>
@@ -5611,11 +6114,15 @@
       <c r="I109" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J109" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J109" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K109" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>147</v>
       </c>
@@ -5643,11 +6150,15 @@
       <c r="I110" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J110" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J110" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K110" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>145</v>
       </c>
@@ -5675,11 +6186,15 @@
       <c r="I111" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J111" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J111" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K111" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>141</v>
       </c>
@@ -5707,11 +6222,15 @@
       <c r="I112" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J112" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J112" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K112" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>138</v>
       </c>
@@ -5724,7 +6243,7 @@
       <c r="D113" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E113" s="1"/>
+      <c r="E113" s="5"/>
       <c r="F113" s="2">
         <v>210.52</v>
       </c>
@@ -5737,11 +6256,15 @@
       <c r="I113" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J113" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J113" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K113" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>136</v>
       </c>
@@ -5769,11 +6292,15 @@
       <c r="I114" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J114" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J114" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K114" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>133</v>
       </c>
@@ -5801,11 +6328,15 @@
       <c r="I115" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J115" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J115" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K115" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>131</v>
       </c>
@@ -5833,11 +6364,15 @@
       <c r="I116" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J116" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J116" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K116" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>128</v>
       </c>
@@ -5865,11 +6400,15 @@
       <c r="I117" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J117" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J117" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K117" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>124</v>
       </c>
@@ -5897,11 +6436,15 @@
       <c r="I118" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J118" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J118" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K118" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>121</v>
       </c>
@@ -5929,11 +6472,15 @@
       <c r="I119" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J119" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J119" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K119" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>118</v>
       </c>
@@ -5958,12 +6505,16 @@
       <c r="H120" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I120" s="1"/>
-      <c r="J120" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I120" s="5"/>
+      <c r="J120" s="5" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K120" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>115</v>
       </c>
@@ -5991,11 +6542,15 @@
       <c r="I121" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J121" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J121" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K121" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>111</v>
       </c>
@@ -6023,11 +6578,15 @@
       <c r="I122" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J122" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J122" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K122" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>109</v>
       </c>
@@ -6055,11 +6614,15 @@
       <c r="I123" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J123" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J123" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K123" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>106</v>
       </c>
@@ -6084,12 +6647,16 @@
       <c r="H124" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="I124" s="1"/>
-      <c r="J124" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I124" s="5"/>
+      <c r="J124" s="5" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K124" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>104</v>
       </c>
@@ -6117,11 +6684,15 @@
       <c r="I125" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J125" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J125" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K125" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>102</v>
       </c>
@@ -6149,11 +6720,15 @@
       <c r="I126" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J126" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J126" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K126" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>97</v>
       </c>
@@ -6181,11 +6756,15 @@
       <c r="I127" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J127" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J127" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K127" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>94</v>
       </c>
@@ -6213,11 +6792,15 @@
       <c r="I128" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J128" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J128" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K128" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>88</v>
       </c>
@@ -6245,11 +6828,15 @@
       <c r="I129" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J129" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J129" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K129" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>85</v>
       </c>
@@ -6277,11 +6864,15 @@
       <c r="I130" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J130" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J130" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K130" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>82</v>
       </c>
@@ -6309,11 +6900,15 @@
       <c r="I131" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J131" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J131" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K131" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>79</v>
       </c>
@@ -6341,11 +6936,15 @@
       <c r="I132" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J132" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J132" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K132" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>75</v>
       </c>
@@ -6373,11 +6972,15 @@
       <c r="I133" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J133" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J133" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K133" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>70</v>
       </c>
@@ -6405,11 +7008,15 @@
       <c r="I134" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J134" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J134" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K134" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>67</v>
       </c>
@@ -6437,11 +7044,15 @@
       <c r="I135" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J135" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J135" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K135" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>65</v>
       </c>
@@ -6469,11 +7080,15 @@
       <c r="I136" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J136" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J136" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K136" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>62</v>
       </c>
@@ -6501,11 +7116,15 @@
       <c r="I137" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J137" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J137" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K137" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>58</v>
       </c>
@@ -6533,11 +7152,15 @@
       <c r="I138" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J138" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J138" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K138" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>54</v>
       </c>
@@ -6565,11 +7188,15 @@
       <c r="I139" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J139" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J139" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K139" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>48</v>
       </c>
@@ -6597,11 +7224,15 @@
       <c r="I140" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J140" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J140" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K140" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>44</v>
       </c>
@@ -6629,11 +7260,15 @@
       <c r="I141" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J141" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J141" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K141" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>41</v>
       </c>
@@ -6661,11 +7296,15 @@
       <c r="I142" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J142" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J142" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K142" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>38</v>
       </c>
@@ -6693,11 +7332,15 @@
       <c r="I143" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J143" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J143" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K143" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>35</v>
       </c>
@@ -6722,12 +7365,16 @@
       <c r="H144" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="I144" s="1"/>
-      <c r="J144" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I144" s="5"/>
+      <c r="J144" s="5" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K144" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>32</v>
       </c>
@@ -6755,11 +7402,15 @@
       <c r="I145" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J145" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J145" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K145" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>29</v>
       </c>
@@ -6787,11 +7438,15 @@
       <c r="I146" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J146" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J146" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K146" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>24</v>
       </c>
@@ -6819,11 +7474,15 @@
       <c r="I147" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J147" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J147" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K147" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>19</v>
       </c>
@@ -6851,11 +7510,15 @@
       <c r="I148" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J148" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J148" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K148" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>14</v>
       </c>
@@ -6883,11 +7546,15 @@
       <c r="I149" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J149" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J149" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K149" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>11</v>
       </c>
@@ -6915,11 +7582,15 @@
       <c r="I150" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J150" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J150" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K150" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>7</v>
       </c>
@@ -6947,7 +7618,11 @@
       <c r="I151" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J151" s="1" t="s">
+      <c r="J151" s="1" t="str">
+        <f>_xlfn.XLOOKUP(TRIM(Table1[[#This Row],[Status2]]),Data_profiling!$A$9:$A$14,Data_profiling!$B$9:$B$14,"Checkmanually")</f>
+        <v>Active</v>
+      </c>
+      <c r="K151" s="1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -6957,4 +7632,121 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79862895-CE92-48DA-A395-9B9682D0B824}">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.26953125" customWidth="1"/>
+    <col min="2" max="2" width="15.1796875" customWidth="1"/>
+    <col min="3" max="3" width="19.1796875" customWidth="1"/>
+    <col min="4" max="4" width="21.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>477</v>
+      </c>
+      <c r="B2" t="s">
+        <v>486</v>
+      </c>
+      <c r="C2">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B3" t="s">
+        <v>486</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>472</v>
+      </c>
+      <c r="B4" t="s">
+        <v>488</v>
+      </c>
+      <c r="D4" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>458</v>
+      </c>
+      <c r="B9" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>429</v>
+      </c>
+      <c r="B11" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>490</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>